<commit_message>
Plan 9 B1: development model and truthful catalog (!166)
## Scope
- EPIC-S8: Development model v2, migration, Excel import, DTO/Gateway/UI freshness rules
- EPIC-S7: server-validated catalog query, SSR pagination, approved secondary facet, truthful bounded aggregates
- Plan 9 v6 approved batch topology and synchronized project canon

## Verification
- Full diff/scope review: PASS
- Local `RISK_SCOPE=schema-data pnpm verify:merge-risky`: PASS at exact head `0fb631f9d0cb729a12db04d808b2f2ed87df3005`
- Native PostgreSQL 18.6 integration: PASS
- Typecheck, architecture and lint: PASS (19 pre-existing lint warnings)

No production, release, tag or mirror.

Co-authored-by: Andrey <chircov.aa@gmail.com>
</commit_message>
<xml_diff>
--- a/fixtures/starter/developments.xlsx
+++ b/fixtures/starter/developments.xlsx
@@ -145,74 +145,81 @@
     <comment ref="I1" authorId="0">
       <text>
         <r>
+          <t>Column districtRaw. Dates use ISO 8601. aliases use | as separator.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0">
+      <text>
+        <r>
           <t>Column address. Dates use ISO 8601. aliases use | as separator.</t>
         </r>
       </text>
     </comment>
-    <comment ref="J1" authorId="0">
+    <comment ref="K1" authorId="0">
       <text>
         <r>
           <t>Column latitude. Dates use ISO 8601. aliases use | as separator.</t>
         </r>
       </text>
     </comment>
-    <comment ref="K1" authorId="0">
+    <comment ref="L1" authorId="0">
       <text>
         <r>
           <t>Column longitude. Dates use ISO 8601. aliases use | as separator.</t>
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0">
+    <comment ref="M1" authorId="0">
       <text>
         <r>
           <t>Column class. Dates use ISO 8601. aliases use | as separator.</t>
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0">
+    <comment ref="N1" authorId="0">
       <text>
         <r>
           <t>Column completion. Dates use ISO 8601. aliases use | as separator.</t>
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="0">
+    <comment ref="O1" authorId="0">
       <text>
         <r>
           <t>Column deadline. Dates use ISO 8601. aliases use | as separator.</t>
         </r>
       </text>
     </comment>
-    <comment ref="O1" authorId="0">
+    <comment ref="P1" authorId="0">
       <text>
         <r>
           <t>Column salesStatus. Dates use ISO 8601. aliases use | as separator.</t>
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="0">
-      <text>
-        <r>
-          <t>Column availability. Dates use ISO 8601. aliases use | as separator.</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="Q1" authorId="0">
       <text>
         <r>
+          <t>Column salesAvailability. Dates use ISO 8601. aliases use | as separator.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="R1" authorId="0">
+      <text>
+        <r>
           <t>Column dataTier. Dates use ISO 8601. aliases use | as separator.</t>
         </r>
       </text>
     </comment>
-    <comment ref="R1" authorId="0">
+    <comment ref="S1" authorId="0">
       <text>
         <r>
           <t>Column status. Dates use ISO 8601. aliases use | as separator.</t>
         </r>
       </text>
     </comment>
-    <comment ref="S1" authorId="0">
+    <comment ref="T1" authorId="0">
       <text>
         <r>
           <t>Column checkedAt. Dates use ISO 8601. aliases use | as separator.</t>
@@ -239,28 +246,35 @@
     <comment ref="B1" authorId="0">
       <text>
         <r>
-          <t>Column label. Dates use ISO 8601. aliases use | as separator.</t>
+          <t>Column roomsLabel. Dates use ISO 8601. aliases use | as separator.</t>
         </r>
       </text>
     </comment>
     <comment ref="C1" authorId="0">
       <text>
         <r>
-          <t>Column amountMinor. Dates use ISO 8601. aliases use | as separator.</t>
+          <t>Column priceFromMinor. Dates use ISO 8601. aliases use | as separator.</t>
         </r>
       </text>
     </comment>
     <comment ref="D1" authorId="0">
       <text>
         <r>
-          <t>Column currency. Dates use ISO 8601. aliases use | as separator.</t>
+          <t>Column priceToMinor. Dates use ISO 8601. aliases use | as separator.</t>
         </r>
       </text>
     </comment>
     <comment ref="E1" authorId="0">
       <text>
         <r>
-          <t>Column checkedAt. Dates use ISO 8601. aliases use | as separator.</t>
+          <t>Column lotsAvailable. Dates use ISO 8601. aliases use | as separator.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0">
+      <text>
+        <r>
+          <t>Column priceCheckedAt. Dates use ISO 8601. aliases use | as separator.</t>
         </r>
       </text>
     </comment>
@@ -305,6 +319,13 @@
     <comment ref="E1" authorId="0">
       <text>
         <r>
+          <t>Column capturedAt. Dates use ISO 8601. aliases use | as separator.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0">
+      <text>
+        <r>
           <t>Column checkedAt. Dates use ISO 8601. aliases use | as separator.</t>
         </r>
       </text>
@@ -352,7 +373,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="81">
   <si>
     <t>slug</t>
   </si>
@@ -429,6 +450,9 @@
     <t>districtSlug</t>
   </si>
   <si>
+    <t>districtRaw</t>
+  </si>
+  <si>
     <t>address</t>
   </si>
   <si>
@@ -450,7 +474,7 @@
     <t>salesStatus</t>
   </si>
   <si>
-    <t>availability</t>
+    <t>salesAvailability</t>
   </si>
   <si>
     <t>dataTier</t>
@@ -486,10 +510,10 @@
     <t>2027-12-31T00:00:00.000Z</t>
   </si>
   <si>
-    <t>available</t>
-  </si>
-  <si>
-    <t>synthetic</t>
+    <t>on_sale</t>
+  </si>
+  <si>
+    <t>confirmed</t>
   </si>
   <si>
     <t>A</t>
@@ -537,22 +561,28 @@
     <t>developmentExternalId</t>
   </si>
   <si>
-    <t>label</t>
-  </si>
-  <si>
-    <t>amountMinor</t>
-  </si>
-  <si>
-    <t>currency</t>
-  </si>
-  <si>
-    <t>от</t>
+    <t>roomsLabel</t>
+  </si>
+  <si>
+    <t>priceFromMinor</t>
+  </si>
+  <si>
+    <t>priceToMinor</t>
+  </si>
+  <si>
+    <t>lotsAvailable</t>
+  </si>
+  <si>
+    <t>priceCheckedAt</t>
+  </si>
+  <si>
+    <t>1-комнатные</t>
   </si>
   <si>
     <t>620000000</t>
   </si>
   <si>
-    <t>RUB</t>
+    <t>1</t>
   </si>
   <si>
     <t>480000000</t>
@@ -568,6 +598,9 @@
   </si>
   <si>
     <t>rights</t>
+  </si>
+  <si>
+    <t>capturedAt</t>
   </si>
   <si>
     <t>text</t>
@@ -1066,13 +1099,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S503"/>
+  <dimension ref="A1:T503"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="19" width="16" customWidth="1"/>
+    <col min="1" max="16" width="16" customWidth="1"/>
+    <col min="17" max="17" width="20" customWidth="1"/>
+    <col min="18" max="20" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>19</v>
       </c>
@@ -1125,51 +1160,54 @@
         <v>33</v>
       </c>
       <c r="R1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="501" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="501" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A501" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B501" t="s">
         <v>8</v>
       </c>
       <c r="C501" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D501" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E501" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F501" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G501" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H501" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I501" t="s">
         <v>41</v>
       </c>
       <c r="J501" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="K501" t="s">
         <v>10</v>
       </c>
       <c r="L501" t="s">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="M501" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="N501" t="s">
         <v>43</v>
@@ -1184,51 +1222,54 @@
         <v>46</v>
       </c>
       <c r="R501" t="s">
+        <v>47</v>
+      </c>
+      <c r="S501" t="s">
         <v>13</v>
       </c>
-      <c r="S501" t="s">
+      <c r="T501" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="502" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="502" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A502" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B502" t="s">
         <v>15</v>
       </c>
       <c r="C502" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D502" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E502" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F502" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G502" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H502" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I502" t="s">
         <v>50</v>
       </c>
       <c r="J502" t="s">
-        <v>10</v>
+        <v>51</v>
       </c>
       <c r="K502" t="s">
         <v>10</v>
       </c>
       <c r="L502" t="s">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="M502" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="N502" t="s">
         <v>43</v>
@@ -1240,54 +1281,57 @@
         <v>45</v>
       </c>
       <c r="Q502" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="R502" t="s">
+        <v>52</v>
+      </c>
+      <c r="S502" t="s">
         <v>13</v>
       </c>
-      <c r="S502" t="s">
+      <c r="T502" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="503" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="503" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A503" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B503" t="s">
         <v>8</v>
       </c>
       <c r="C503" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D503" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E503" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F503" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G503" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H503" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I503" t="s">
         <v>58</v>
       </c>
       <c r="J503" t="s">
-        <v>10</v>
+        <v>59</v>
       </c>
       <c r="K503" t="s">
         <v>10</v>
       </c>
       <c r="L503" t="s">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="M503" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="N503" t="s">
         <v>43</v>
@@ -1299,39 +1343,48 @@
         <v>45</v>
       </c>
       <c r="Q503" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="R503" t="s">
+        <v>60</v>
+      </c>
+      <c r="S503" t="s">
         <v>13</v>
       </c>
-      <c r="S503" t="s">
+      <c r="T503" t="s">
         <v>14</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="8">
+  <dataValidations count="10">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: residential_complex, cottage_village" sqref="E10:E500">
       <formula1>"residential_complex,cottage_village"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: residential_complex, cottage_village" sqref="E2:E500">
       <formula1>"residential_complex,cottage_village"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: available, limited, sold_out, paused" sqref="O10:O500">
-      <formula1>"available,limited,sold_out,paused"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: on_sale, sales_finished, completed" sqref="P10:P500">
+      <formula1>"on_sale,sales_finished,completed"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: available, limited, sold_out, paused" sqref="O2:O500">
-      <formula1>"available,limited,sold_out,paused"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: on_sale, sales_finished, completed" sqref="P2:P500">
+      <formula1>"on_sale,sales_finished,completed"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: A, B, C" sqref="Q10:Q500">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: in_inventory, confirmed, none" sqref="Q10:Q500">
+      <formula1>"in_inventory,confirmed,none"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: in_inventory, confirmed, none" sqref="Q2:Q500">
+      <formula1>"in_inventory,confirmed,none"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: A, B, C" sqref="R10:R500">
       <formula1>"A,B,C"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: A, B, C" sqref="Q2:Q500">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: A, B, C" sqref="R2:R500">
       <formula1>"A,B,C"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: draft, published, archived" sqref="R10:R500">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: draft, published, archived" sqref="S10:S500">
       <formula1>"draft,published,archived"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: draft, published, archived" sqref="R2:R500">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: draft, published, archived" sqref="S2:S500">
       <formula1>"draft,published,archived"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1343,90 +1396,97 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E503"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="5" width="16" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="4" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>7</v>
+        <v>65</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>66</v>
       </c>
     </row>
-    <row r="501" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A501" t="s">
-        <v>34</v>
-      </c>
-      <c r="B501" t="s">
-        <v>64</v>
-      </c>
-      <c r="C501" t="s">
-        <v>65</v>
-      </c>
-      <c r="D501" t="s">
-        <v>66</v>
-      </c>
-      <c r="E501" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="502" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A502" t="s">
-        <v>47</v>
-      </c>
-      <c r="B502" t="s">
-        <v>64</v>
-      </c>
-      <c r="C502" t="s">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" t="s">
         <v>67</v>
       </c>
-      <c r="D502" t="s">
-        <v>66</v>
-      </c>
-      <c r="E502" t="s">
+      <c r="C3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3" t="s">
+        <v>69</v>
+      </c>
+      <c r="F3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="503" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A503" t="s">
-        <v>52</v>
-      </c>
-      <c r="B503" t="s">
-        <v>64</v>
-      </c>
-      <c r="C503" t="s">
-        <v>68</v>
-      </c>
-      <c r="D503" t="s">
-        <v>66</v>
-      </c>
-      <c r="E503" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F4" t="s">
         <v>14</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: RUB" sqref="D10:D500">
-      <formula1>"RUB"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: RUB" sqref="D2:D500">
-      <formula1>"RUB"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <legacyDrawing r:id="rId2"/>
@@ -1435,37 +1495,40 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="5" width="16" customWidth="1"/>
+    <col min="2" max="6" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: image, plan, document" sqref="C10:C500">
-      <formula1>"image,plan,document"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: hero, gallery, layout, construction_progress, document, video" sqref="C10:C500">
+      <formula1>"hero,gallery,layout,construction_progress,document,video"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: image, plan, document" sqref="C2:C500">
-      <formula1>"image,plan,document"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Allowed values: hero, gallery, layout, construction_progress, document, video" sqref="C2:C500">
+      <formula1>"hero,gallery,layout,construction_progress,document,video"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1485,13 +1548,13 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>7</v>
@@ -1499,13 +1562,13 @@
     </row>
     <row r="501" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A501" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B501" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C501" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D501" t="s">
         <v>14</v>
@@ -1513,13 +1576,13 @@
     </row>
     <row r="502" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A502" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B502" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C502" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D502" t="s">
         <v>14</v>
@@ -1527,13 +1590,13 @@
     </row>
     <row r="503" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A503" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B503" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C503" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D503" t="s">
         <v>14</v>

</xml_diff>